<commit_message>
Añadimos imagenes al RAG
</commit_message>
<xml_diff>
--- a/Local/faqs.xlsx
+++ b/Local/faqs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Downloads\Tesis\Local\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D09906CF-F33C-448F-AEEE-76FF422916E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8454752F-BE5C-4E20-845A-1188B4D5C8DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="57">
   <si>
     <t>type</t>
   </si>
@@ -353,18 +353,34 @@
       <t>. 🏞️🔥</t>
     </r>
   </si>
+  <si>
+    <t>img</t>
+  </si>
+  <si>
+    <t>¿Cuál es el proceso de inscripción de la Rio21k?</t>
+  </si>
+  <si>
+    <t>imagenes\inscripcion_rio21k.jpg</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -425,16 +441,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -632,7 +651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.21875" style="1" customWidth="1"/>
@@ -927,6 +946,17 @@
         <v>47</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>